<commit_message>
feat(consumption): correct MACRO consumption for excluded emissions
</commit_message>
<xml_diff>
--- a/Manuscript/Tables/SI_text_numbers.xlsx
+++ b/Manuscript/Tables/SI_text_numbers.xlsx
@@ -882,16 +882,16 @@
         <v>-0.7831959098277558</v>
       </c>
       <c r="C2">
-        <v>-1.039212373692243</v>
+        <v>-0.8162042843561071</v>
       </c>
       <c r="D2">
-        <v>-1.255817593868411</v>
+        <v>-1.032075797719282</v>
       </c>
       <c r="E2">
-        <v>-0.2580374022446938</v>
+        <v>-0.03326893547019716</v>
       </c>
       <c r="F2">
-        <v>-0.476352457000245</v>
+        <v>-0.250844491690474</v>
       </c>
     </row>
     <row r="3">
@@ -904,16 +904,16 @@
         <v>-0.7831959098277558</v>
       </c>
       <c r="C3">
-        <v>-1.013749180112423</v>
+        <v>-0.7907143602818875</v>
       </c>
       <c r="D3">
-        <v>-1.527742334734132</v>
+        <v>-1.303840527901801</v>
       </c>
       <c r="E3">
-        <v>-0.2323732077432483</v>
+        <v>-0.007577799469632883</v>
       </c>
       <c r="F3">
-        <v>-0.7504237127308623</v>
+        <v>-0.5247544736482971</v>
       </c>
     </row>
     <row r="4">
@@ -926,16 +926,16 @@
         <v>-0.7831959098277558</v>
       </c>
       <c r="C4">
-        <v>-1.008825798422962</v>
+        <v>-0.7858119114797637</v>
       </c>
       <c r="D4">
-        <v>-1.334649083597818</v>
+        <v>-1.109091645237009</v>
       </c>
       <c r="E4">
-        <v>-0.2274109619476801</v>
+        <v>-0.002636651801070434</v>
       </c>
       <c r="F4">
-        <v>-0.555806225393916</v>
+        <v>-0.3284682855870519</v>
       </c>
     </row>
     <row r="5">
@@ -948,16 +948,16 @@
         <v>-0.7831959098277558</v>
       </c>
       <c r="C5">
-        <v>-1.014081144807741</v>
+        <v>-0.7911226310180877</v>
       </c>
       <c r="D5">
-        <v>-1.325297700495919</v>
+        <v>-1.099721669897897</v>
       </c>
       <c r="E5">
-        <v>-0.2327077928957957</v>
+        <v>-0.007989293006382077</v>
       </c>
       <c r="F5">
-        <v>-0.5463810245041543</v>
+        <v>-0.3190243456969945</v>
       </c>
     </row>
     <row r="6">
@@ -970,16 +970,16 @@
         <v>-0.7831959098277558</v>
       </c>
       <c r="C6">
-        <v>-1.005575808516155</v>
+        <v>-0.7825169955499158</v>
       </c>
       <c r="D6">
-        <v>-1.061185725447701</v>
+        <v>-0.8380803689188605</v>
       </c>
       <c r="E6">
-        <v>-0.2241353173261773</v>
+        <v>0.0006842734797452915</v>
       </c>
       <c r="F6">
-        <v>-0.2801842068681196</v>
+        <v>-0.05531770509481793</v>
       </c>
     </row>
     <row r="7">
@@ -992,16 +992,16 @@
         <v>-1.348674277434335</v>
       </c>
       <c r="C7">
-        <v>-1.995694779170654</v>
+        <v>-1.40495372883638</v>
       </c>
       <c r="D7">
-        <v>-1.964451156237398</v>
+        <v>-1.373089928047217</v>
       </c>
       <c r="E7">
-        <v>-0.6558659977423078</v>
+        <v>-0.05704885463001124</v>
       </c>
       <c r="F7">
-        <v>-0.6241952394383372</v>
+        <v>-0.02474943994320514</v>
       </c>
     </row>
     <row r="8">
@@ -1014,16 +1014,16 @@
         <v>-0.7831959098277558</v>
       </c>
       <c r="C8">
-        <v>-1.004006224210178</v>
+        <v>-0.7809484821158152</v>
       </c>
       <c r="D8">
-        <v>-1.147192396237507</v>
+        <v>-0.9226746108650603</v>
       </c>
       <c r="E8">
-        <v>-0.222553343062473</v>
+        <v>0.002265168418343684</v>
       </c>
       <c r="F8">
-        <v>-0.3668697956436259</v>
+        <v>-0.1405797156200887</v>
       </c>
     </row>
     <row r="9">
@@ -1036,16 +1036,16 @@
         <v>-0.7831959098277558</v>
       </c>
       <c r="C9">
-        <v>-1.644646564752747</v>
+        <v>-1.421059704506613</v>
       </c>
       <c r="D9">
-        <v>-1.64129645184555</v>
+        <v>-1.417663976914055</v>
       </c>
       <c r="E9">
-        <v>-0.8682507593593416</v>
+        <v>-0.6428989529829455</v>
       </c>
       <c r="F9">
-        <v>-0.8648742013882221</v>
+        <v>-0.6394764202540418</v>
       </c>
     </row>
   </sheetData>

</xml_diff>